<commit_message>
Add new psi_planning tool
</commit_message>
<xml_diff>
--- a/docs/dummy_psi.xlsx
+++ b/docs/dummy_psi.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28440" windowHeight="14020"/>
+    <workbookView windowWidth="28400" windowHeight="14020"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1312,12 +1312,12 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <f ca="1">IF(B4*3&gt;B5,B4*3-B5,0)</f>
+        <f ca="1">IF(C4*3&gt;B5,C4*3-B5,0)</f>
         <v>0</v>
       </c>
       <c r="C3">
-        <f ca="1" t="shared" ref="C3:AE3" si="0">IF(C4*3&gt;C5,C4*3-C5,0)</f>
-        <v>63</v>
+        <f ca="1" t="shared" ref="C3:AE3" si="0">IF(D4*3&gt;C5,D4*3-C5,0)</f>
+        <v>0</v>
       </c>
       <c r="D3">
         <f ca="1" t="shared" si="0"/>
@@ -1325,79 +1325,79 @@
       </c>
       <c r="E3">
         <f ca="1" t="shared" si="0"/>
-        <v>9</v>
+        <v>117</v>
       </c>
       <c r="F3">
         <f ca="1" t="shared" si="0"/>
-        <v>92</v>
+        <v>0</v>
       </c>
       <c r="G3">
         <f ca="1" t="shared" si="0"/>
-        <v>99</v>
+        <v>50</v>
       </c>
       <c r="H3">
         <f ca="1" t="shared" si="0"/>
-        <v>173</v>
+        <v>68</v>
       </c>
       <c r="I3">
         <f ca="1" t="shared" si="0"/>
+        <v>103</v>
+      </c>
+      <c r="J3">
+        <f ca="1" t="shared" si="0"/>
+        <v>112</v>
+      </c>
+      <c r="K3">
+        <f ca="1" t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="L3">
+        <f ca="1" t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="M3">
+        <f ca="1" t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="N3">
+        <f ca="1" t="shared" si="0"/>
+        <v>144</v>
+      </c>
+      <c r="O3">
+        <f ca="1" t="shared" si="0"/>
+        <v>150</v>
+      </c>
+      <c r="P3">
+        <f ca="1" t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="Q3">
+        <f ca="1" t="shared" si="0"/>
+        <v>60</v>
+      </c>
+      <c r="R3">
+        <f ca="1" t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="S3">
+        <f ca="1" t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="T3">
+        <f ca="1" t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="U3">
+        <f ca="1" t="shared" si="0"/>
+        <v>70</v>
+      </c>
+      <c r="V3">
+        <f ca="1" t="shared" si="0"/>
         <v>87</v>
       </c>
-      <c r="J3">
-        <f ca="1" t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="K3">
-        <f ca="1" t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="L3">
-        <f ca="1" t="shared" si="0"/>
-        <v>148</v>
-      </c>
-      <c r="M3">
-        <f ca="1" t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="N3">
-        <f ca="1" t="shared" si="0"/>
-        <v>21</v>
-      </c>
-      <c r="O3">
-        <f ca="1" t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="P3">
-        <f ca="1" t="shared" si="0"/>
-        <v>135</v>
-      </c>
-      <c r="Q3">
-        <f ca="1" t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="R3">
-        <f ca="1" t="shared" si="0"/>
-        <v>47</v>
-      </c>
-      <c r="S3">
-        <f ca="1" t="shared" si="0"/>
-        <v>3</v>
-      </c>
-      <c r="T3">
-        <f ca="1" t="shared" si="0"/>
-        <v>142</v>
-      </c>
-      <c r="U3">
-        <f ca="1" t="shared" si="0"/>
-        <v>103</v>
-      </c>
-      <c r="V3">
-        <f ca="1" t="shared" si="0"/>
-        <v>28</v>
-      </c>
       <c r="W3">
         <f ca="1" t="shared" si="0"/>
-        <v>0</v>
+        <v>115</v>
       </c>
       <c r="X3">
         <f ca="1" t="shared" si="0"/>
@@ -1405,27 +1405,27 @@
       </c>
       <c r="Y3">
         <f ca="1" t="shared" si="0"/>
-        <v>233</v>
+        <v>0</v>
       </c>
       <c r="Z3">
         <f ca="1" t="shared" si="0"/>
-        <v>0</v>
+        <v>138</v>
       </c>
       <c r="AA3">
         <f ca="1" t="shared" si="0"/>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AB3">
         <f ca="1" t="shared" si="0"/>
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="AC3">
         <f ca="1" t="shared" si="0"/>
-        <v>96</v>
+        <v>210</v>
       </c>
       <c r="AD3">
         <f ca="1" t="shared" si="0"/>
-        <v>136</v>
+        <v>0</v>
       </c>
       <c r="AE3">
         <f ca="1" t="shared" si="0"/>
@@ -1438,123 +1438,123 @@
       </c>
       <c r="B4">
         <f ca="1">RANDBETWEEN(10,100)</f>
-        <v>31</v>
+        <v>82</v>
       </c>
       <c r="C4">
         <f ca="1" t="shared" ref="C4:L4" si="1">RANDBETWEEN(10,100)</f>
-        <v>66</v>
+        <v>11</v>
       </c>
       <c r="D4">
         <f ca="1" t="shared" si="1"/>
-        <v>15</v>
+        <v>47</v>
       </c>
       <c r="E4">
         <f ca="1" t="shared" si="1"/>
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F4">
         <f ca="1" t="shared" si="1"/>
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="G4">
         <f ca="1" t="shared" si="1"/>
-        <v>69</v>
+        <v>33</v>
       </c>
       <c r="H4">
         <f ca="1" t="shared" si="1"/>
-        <v>95</v>
+        <v>53</v>
       </c>
       <c r="I4">
         <f ca="1" t="shared" si="1"/>
-        <v>93</v>
+        <v>58</v>
       </c>
       <c r="J4">
         <f ca="1" t="shared" si="1"/>
-        <v>36</v>
+        <v>73</v>
       </c>
       <c r="K4">
         <f ca="1" t="shared" si="1"/>
-        <v>31</v>
+        <v>86</v>
       </c>
       <c r="L4">
         <f ca="1" t="shared" si="1"/>
-        <v>90</v>
+        <v>64</v>
       </c>
       <c r="M4">
         <f ca="1" t="shared" ref="M4:V4" si="2">RANDBETWEEN(10,100)</f>
-        <v>51</v>
+        <v>24</v>
       </c>
       <c r="N4">
         <f ca="1" t="shared" si="2"/>
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="O4">
         <f ca="1" t="shared" si="2"/>
-        <v>15</v>
+        <v>72</v>
       </c>
       <c r="P4">
         <f ca="1" t="shared" si="2"/>
-        <v>75</v>
+        <v>98</v>
       </c>
       <c r="Q4">
         <f ca="1" t="shared" si="2"/>
-        <v>52</v>
+        <v>10</v>
       </c>
       <c r="R4">
         <f ca="1" t="shared" si="2"/>
-        <v>55</v>
+        <v>82</v>
       </c>
       <c r="S4">
         <f ca="1" t="shared" si="2"/>
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="T4">
         <f ca="1" t="shared" si="2"/>
-        <v>67</v>
+        <v>16</v>
       </c>
       <c r="U4">
         <f ca="1" t="shared" si="2"/>
-        <v>76</v>
+        <v>37</v>
       </c>
       <c r="V4">
         <f ca="1" t="shared" si="2"/>
-        <v>64</v>
+        <v>48</v>
       </c>
       <c r="W4">
         <f ca="1" t="shared" ref="W4:AE4" si="3">RANDBETWEEN(10,100)</f>
-        <v>18</v>
+        <v>61</v>
       </c>
       <c r="X4">
         <f ca="1" t="shared" si="3"/>
-        <v>11</v>
+        <v>79</v>
       </c>
       <c r="Y4">
         <f ca="1" t="shared" si="3"/>
-        <v>99</v>
+        <v>29</v>
       </c>
       <c r="Z4">
         <f ca="1" t="shared" si="3"/>
-        <v>53</v>
+        <v>33</v>
       </c>
       <c r="AA4">
         <f ca="1" t="shared" si="3"/>
-        <v>33</v>
+        <v>78</v>
       </c>
       <c r="AB4">
         <f ca="1" t="shared" si="3"/>
-        <v>35</v>
+        <v>54</v>
       </c>
       <c r="AC4">
         <f ca="1" t="shared" si="3"/>
-        <v>68</v>
+        <v>42</v>
       </c>
       <c r="AD4">
         <f ca="1" t="shared" si="3"/>
-        <v>85</v>
+        <v>98</v>
       </c>
       <c r="AE4">
         <f ca="1" t="shared" si="3"/>
-        <v>30</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5" spans="1:31">
@@ -1566,119 +1566,119 @@
       </c>
       <c r="C5">
         <f ca="1">B5-C4+B3</f>
-        <v>135</v>
+        <v>190</v>
       </c>
       <c r="D5">
         <f ca="1" t="shared" ref="D5:AE5" si="4">C5-D4+C3</f>
-        <v>183</v>
+        <v>143</v>
       </c>
       <c r="E5">
         <f ca="1" t="shared" si="4"/>
-        <v>135</v>
+        <v>96</v>
       </c>
       <c r="F5">
         <f ca="1" t="shared" si="4"/>
-        <v>85</v>
+        <v>142</v>
       </c>
       <c r="G5">
         <f ca="1" t="shared" si="4"/>
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H5">
         <f ca="1" t="shared" si="4"/>
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="I5">
         <f ca="1" t="shared" si="4"/>
-        <v>192</v>
+        <v>116</v>
       </c>
       <c r="J5">
         <f ca="1" t="shared" si="4"/>
-        <v>243</v>
+        <v>146</v>
       </c>
       <c r="K5">
         <f ca="1" t="shared" si="4"/>
-        <v>212</v>
+        <v>172</v>
       </c>
       <c r="L5">
         <f ca="1" t="shared" si="4"/>
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="M5">
         <f ca="1" t="shared" si="4"/>
-        <v>219</v>
+        <v>104</v>
       </c>
       <c r="N5">
         <f ca="1" t="shared" si="4"/>
-        <v>159</v>
+        <v>72</v>
       </c>
       <c r="O5">
         <f ca="1" t="shared" si="4"/>
-        <v>165</v>
+        <v>144</v>
       </c>
       <c r="P5">
         <f ca="1" t="shared" si="4"/>
-        <v>90</v>
+        <v>196</v>
       </c>
       <c r="Q5">
         <f ca="1" t="shared" si="4"/>
-        <v>173</v>
+        <v>186</v>
       </c>
       <c r="R5">
         <f ca="1" t="shared" si="4"/>
-        <v>118</v>
+        <v>164</v>
       </c>
       <c r="S5">
         <f ca="1" t="shared" si="4"/>
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="T5">
         <f ca="1" t="shared" si="4"/>
-        <v>59</v>
+        <v>103</v>
       </c>
       <c r="U5">
         <f ca="1" t="shared" si="4"/>
-        <v>125</v>
+        <v>74</v>
       </c>
       <c r="V5">
         <f ca="1" t="shared" si="4"/>
-        <v>164</v>
+        <v>96</v>
       </c>
       <c r="W5">
         <f ca="1" t="shared" si="4"/>
-        <v>174</v>
+        <v>122</v>
       </c>
       <c r="X5">
         <f ca="1" t="shared" si="4"/>
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="Y5">
         <f ca="1" t="shared" si="4"/>
-        <v>64</v>
+        <v>129</v>
       </c>
       <c r="Z5">
         <f ca="1" t="shared" si="4"/>
-        <v>244</v>
+        <v>96</v>
       </c>
       <c r="AA5">
         <f ca="1" t="shared" si="4"/>
-        <v>211</v>
+        <v>156</v>
       </c>
       <c r="AB5">
         <f ca="1" t="shared" si="4"/>
-        <v>176</v>
+        <v>108</v>
       </c>
       <c r="AC5">
         <f ca="1" t="shared" si="4"/>
-        <v>108</v>
+        <v>84</v>
       </c>
       <c r="AD5">
         <f ca="1" t="shared" si="4"/>
-        <v>119</v>
+        <v>196</v>
       </c>
       <c r="AE5">
         <f ca="1" t="shared" si="4"/>
-        <v>225</v>
+        <v>160</v>
       </c>
     </row>
     <row r="6" spans="1:31">
@@ -1792,8 +1792,8 @@
         <v>2</v>
       </c>
       <c r="B10">
-        <f ca="1" t="shared" ref="B10:AE10" si="5">IF(B11*3&gt;B12,B11*3-B12,0)</f>
-        <v>164</v>
+        <f ca="1" t="shared" ref="B10:AE10" si="5">IF(C11*3&gt;B12,C11*3-B12,0)</f>
+        <v>191</v>
       </c>
       <c r="C10">
         <f ca="1" t="shared" si="5"/>
@@ -1805,11 +1805,11 @@
       </c>
       <c r="E10">
         <f ca="1" t="shared" si="5"/>
-        <v>177</v>
+        <v>0</v>
       </c>
       <c r="F10">
         <f ca="1" t="shared" si="5"/>
-        <v>122</v>
+        <v>185</v>
       </c>
       <c r="G10">
         <f ca="1" t="shared" si="5"/>
@@ -1817,15 +1817,15 @@
       </c>
       <c r="H10">
         <f ca="1" t="shared" si="5"/>
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="I10">
         <f ca="1" t="shared" si="5"/>
-        <v>0</v>
+        <v>114</v>
       </c>
       <c r="J10">
         <f ca="1" t="shared" si="5"/>
-        <v>161</v>
+        <v>0</v>
       </c>
       <c r="K10">
         <f ca="1" t="shared" si="5"/>
@@ -1833,15 +1833,15 @@
       </c>
       <c r="L10">
         <f ca="1" t="shared" si="5"/>
-        <v>146</v>
+        <v>0</v>
       </c>
       <c r="M10">
         <f ca="1" t="shared" si="5"/>
-        <v>0</v>
+        <v>44</v>
       </c>
       <c r="N10">
         <f ca="1" t="shared" si="5"/>
-        <v>66</v>
+        <v>186</v>
       </c>
       <c r="O10">
         <f ca="1" t="shared" si="5"/>
@@ -1849,11 +1849,11 @@
       </c>
       <c r="P10">
         <f ca="1" t="shared" si="5"/>
-        <v>0</v>
+        <v>77</v>
       </c>
       <c r="Q10">
         <f ca="1" t="shared" si="5"/>
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="R10">
         <f ca="1" t="shared" si="5"/>
@@ -1861,15 +1861,15 @@
       </c>
       <c r="S10">
         <f ca="1" t="shared" si="5"/>
-        <v>31</v>
+        <v>136</v>
       </c>
       <c r="T10">
         <f ca="1" t="shared" si="5"/>
-        <v>202</v>
+        <v>0</v>
       </c>
       <c r="U10">
         <f ca="1" t="shared" si="5"/>
-        <v>0</v>
+        <v>79</v>
       </c>
       <c r="V10">
         <f ca="1" t="shared" si="5"/>
@@ -1881,23 +1881,23 @@
       </c>
       <c r="X10">
         <f ca="1" t="shared" si="5"/>
-        <v>105</v>
+        <v>195</v>
       </c>
       <c r="Y10">
         <f ca="1" t="shared" si="5"/>
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="Z10">
         <f ca="1" t="shared" si="5"/>
-        <v>177</v>
+        <v>0</v>
       </c>
       <c r="AA10">
         <f ca="1" t="shared" si="5"/>
-        <v>61</v>
+        <v>130</v>
       </c>
       <c r="AB10">
         <f ca="1" t="shared" si="5"/>
-        <v>132</v>
+        <v>84</v>
       </c>
       <c r="AC10">
         <f ca="1" t="shared" si="5"/>
@@ -1905,7 +1905,7 @@
       </c>
       <c r="AD10">
         <f ca="1" t="shared" si="5"/>
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="AE10">
         <f ca="1" t="shared" si="5"/>
@@ -1918,123 +1918,123 @@
       </c>
       <c r="B11">
         <f ca="1" t="shared" ref="B11:AE11" si="6">RANDBETWEEN(10,100)</f>
-        <v>78</v>
+        <v>11</v>
       </c>
       <c r="C11">
         <f ca="1" t="shared" si="6"/>
-        <v>33</v>
+        <v>87</v>
       </c>
       <c r="D11">
         <f ca="1" t="shared" si="6"/>
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="E11">
         <f ca="1" t="shared" si="6"/>
-        <v>86</v>
+        <v>30</v>
       </c>
       <c r="F11">
         <f ca="1" t="shared" si="6"/>
-        <v>95</v>
+        <v>21</v>
       </c>
       <c r="G11">
         <f ca="1" t="shared" si="6"/>
+        <v>90</v>
+      </c>
+      <c r="H11">
+        <f ca="1" t="shared" si="6"/>
+        <v>11</v>
+      </c>
+      <c r="I11">
+        <f ca="1" t="shared" si="6"/>
+        <v>63</v>
+      </c>
+      <c r="J11">
+        <f ca="1" t="shared" si="6"/>
+        <v>80</v>
+      </c>
+      <c r="K11">
+        <f ca="1" t="shared" si="6"/>
+        <v>16</v>
+      </c>
+      <c r="L11">
+        <f ca="1" t="shared" si="6"/>
+        <v>13</v>
+      </c>
+      <c r="M11">
+        <f ca="1" t="shared" si="6"/>
+        <v>22</v>
+      </c>
+      <c r="N11">
+        <f ca="1" t="shared" si="6"/>
+        <v>51</v>
+      </c>
+      <c r="O11">
+        <f ca="1" t="shared" si="6"/>
+        <v>96</v>
+      </c>
+      <c r="P11">
+        <f ca="1" t="shared" si="6"/>
+        <v>59</v>
+      </c>
+      <c r="Q11">
+        <f ca="1" t="shared" si="6"/>
+        <v>70</v>
+      </c>
+      <c r="R11">
+        <f ca="1" t="shared" si="6"/>
+        <v>17</v>
+      </c>
+      <c r="S11">
+        <f ca="1" t="shared" si="6"/>
+        <v>19</v>
+      </c>
+      <c r="T11">
+        <f ca="1" t="shared" si="6"/>
+        <v>80</v>
+      </c>
+      <c r="U11">
+        <f ca="1" t="shared" si="6"/>
+        <v>44</v>
+      </c>
+      <c r="V11">
+        <f ca="1" t="shared" si="6"/>
         <v>65</v>
       </c>
-      <c r="H11">
+      <c r="W11">
+        <f ca="1" t="shared" si="6"/>
+        <v>43</v>
+      </c>
+      <c r="X11">
+        <f ca="1" t="shared" si="6"/>
+        <v>27</v>
+      </c>
+      <c r="Y11">
+        <f ca="1" t="shared" si="6"/>
+        <v>85</v>
+      </c>
+      <c r="Z11">
+        <f ca="1" t="shared" si="6"/>
+        <v>66</v>
+      </c>
+      <c r="AA11">
+        <f ca="1" t="shared" si="6"/>
+        <v>10</v>
+      </c>
+      <c r="AB11">
+        <f ca="1" t="shared" si="6"/>
+        <v>84</v>
+      </c>
+      <c r="AC11">
+        <f ca="1" t="shared" si="6"/>
+        <v>84</v>
+      </c>
+      <c r="AD11">
+        <f ca="1" t="shared" si="6"/>
+        <v>56</v>
+      </c>
+      <c r="AE11">
         <f ca="1" t="shared" si="6"/>
         <v>42</v>
-      </c>
-      <c r="I11">
-        <f ca="1" t="shared" si="6"/>
-        <v>19</v>
-      </c>
-      <c r="J11">
-        <f ca="1" t="shared" si="6"/>
-        <v>80</v>
-      </c>
-      <c r="K11">
-        <f ca="1" t="shared" si="6"/>
-        <v>18</v>
-      </c>
-      <c r="L11">
-        <f ca="1" t="shared" si="6"/>
-        <v>92</v>
-      </c>
-      <c r="M11">
-        <f ca="1" t="shared" si="6"/>
-        <v>50</v>
-      </c>
-      <c r="N11">
-        <f ca="1" t="shared" si="6"/>
-        <v>73</v>
-      </c>
-      <c r="O11">
-        <f ca="1" t="shared" si="6"/>
-        <v>46</v>
-      </c>
-      <c r="P11">
-        <f ca="1" t="shared" si="6"/>
-        <v>43</v>
-      </c>
-      <c r="Q11">
-        <f ca="1" t="shared" si="6"/>
-        <v>45</v>
-      </c>
-      <c r="R11">
-        <f ca="1" t="shared" si="6"/>
-        <v>14</v>
-      </c>
-      <c r="S11">
-        <f ca="1" t="shared" si="6"/>
-        <v>38</v>
-      </c>
-      <c r="T11">
-        <f ca="1" t="shared" si="6"/>
-        <v>79</v>
-      </c>
-      <c r="U11">
-        <f ca="1" t="shared" si="6"/>
-        <v>47</v>
-      </c>
-      <c r="V11">
-        <f ca="1" t="shared" si="6"/>
-        <v>14</v>
-      </c>
-      <c r="W11">
-        <f ca="1" t="shared" si="6"/>
-        <v>37</v>
-      </c>
-      <c r="X11">
-        <f ca="1" t="shared" si="6"/>
-        <v>61</v>
-      </c>
-      <c r="Y11">
-        <f ca="1" t="shared" si="6"/>
-        <v>36</v>
-      </c>
-      <c r="Z11">
-        <f ca="1" t="shared" si="6"/>
-        <v>81</v>
-      </c>
-      <c r="AA11">
-        <f ca="1" t="shared" si="6"/>
-        <v>76</v>
-      </c>
-      <c r="AB11">
-        <f ca="1" t="shared" si="6"/>
-        <v>90</v>
-      </c>
-      <c r="AC11">
-        <f ca="1" t="shared" si="6"/>
-        <v>51</v>
-      </c>
-      <c r="AD11">
-        <f ca="1" t="shared" si="6"/>
-        <v>88</v>
-      </c>
-      <c r="AE11">
-        <f ca="1" t="shared" si="6"/>
-        <v>51</v>
       </c>
     </row>
     <row r="12" spans="1:31">
@@ -2046,119 +2046,119 @@
       </c>
       <c r="C12">
         <f ca="1" t="shared" ref="C12:AE12" si="7">B12-C11+B10</f>
-        <v>201</v>
+        <v>174</v>
       </c>
       <c r="D12">
         <f ca="1" t="shared" si="7"/>
-        <v>167</v>
+        <v>136</v>
       </c>
       <c r="E12">
         <f ca="1" t="shared" si="7"/>
-        <v>81</v>
+        <v>106</v>
       </c>
       <c r="F12">
         <f ca="1" t="shared" si="7"/>
-        <v>163</v>
+        <v>85</v>
       </c>
       <c r="G12">
         <f ca="1" t="shared" si="7"/>
-        <v>220</v>
+        <v>180</v>
       </c>
       <c r="H12">
         <f ca="1" t="shared" si="7"/>
-        <v>178</v>
+        <v>169</v>
       </c>
       <c r="I12">
         <f ca="1" t="shared" si="7"/>
-        <v>159</v>
+        <v>126</v>
       </c>
       <c r="J12">
         <f ca="1" t="shared" si="7"/>
-        <v>79</v>
+        <v>160</v>
       </c>
       <c r="K12">
         <f ca="1" t="shared" si="7"/>
-        <v>222</v>
+        <v>144</v>
       </c>
       <c r="L12">
         <f ca="1" t="shared" si="7"/>
+        <v>131</v>
+      </c>
+      <c r="M12">
+        <f ca="1" t="shared" si="7"/>
+        <v>109</v>
+      </c>
+      <c r="N12">
+        <f ca="1" t="shared" si="7"/>
+        <v>102</v>
+      </c>
+      <c r="O12">
+        <f ca="1" t="shared" si="7"/>
+        <v>192</v>
+      </c>
+      <c r="P12">
+        <f ca="1" t="shared" si="7"/>
+        <v>133</v>
+      </c>
+      <c r="Q12">
+        <f ca="1" t="shared" si="7"/>
+        <v>140</v>
+      </c>
+      <c r="R12">
+        <f ca="1" t="shared" si="7"/>
+        <v>123</v>
+      </c>
+      <c r="S12">
+        <f ca="1" t="shared" si="7"/>
+        <v>104</v>
+      </c>
+      <c r="T12">
+        <f ca="1" t="shared" si="7"/>
+        <v>160</v>
+      </c>
+      <c r="U12">
+        <f ca="1" t="shared" si="7"/>
+        <v>116</v>
+      </c>
+      <c r="V12">
+        <f ca="1" t="shared" si="7"/>
         <v>130</v>
       </c>
-      <c r="M12">
-        <f ca="1" t="shared" si="7"/>
-        <v>226</v>
-      </c>
-      <c r="N12">
-        <f ca="1" t="shared" si="7"/>
-        <v>153</v>
-      </c>
-      <c r="O12">
-        <f ca="1" t="shared" si="7"/>
-        <v>173</v>
-      </c>
-      <c r="P12">
-        <f ca="1" t="shared" si="7"/>
-        <v>130</v>
-      </c>
-      <c r="Q12">
-        <f ca="1" t="shared" si="7"/>
-        <v>85</v>
-      </c>
-      <c r="R12">
-        <f ca="1" t="shared" si="7"/>
-        <v>121</v>
-      </c>
-      <c r="S12">
-        <f ca="1" t="shared" si="7"/>
-        <v>83</v>
-      </c>
-      <c r="T12">
-        <f ca="1" t="shared" si="7"/>
-        <v>35</v>
-      </c>
-      <c r="U12">
-        <f ca="1" t="shared" si="7"/>
-        <v>190</v>
-      </c>
-      <c r="V12">
-        <f ca="1" t="shared" si="7"/>
-        <v>176</v>
-      </c>
       <c r="W12">
         <f ca="1" t="shared" si="7"/>
-        <v>139</v>
+        <v>87</v>
       </c>
       <c r="X12">
         <f ca="1" t="shared" si="7"/>
-        <v>78</v>
+        <v>60</v>
       </c>
       <c r="Y12">
         <f ca="1" t="shared" si="7"/>
-        <v>147</v>
+        <v>170</v>
       </c>
       <c r="Z12">
         <f ca="1" t="shared" si="7"/>
-        <v>66</v>
+        <v>132</v>
       </c>
       <c r="AA12">
         <f ca="1" t="shared" si="7"/>
-        <v>167</v>
+        <v>122</v>
       </c>
       <c r="AB12">
         <f ca="1" t="shared" si="7"/>
-        <v>138</v>
+        <v>168</v>
       </c>
       <c r="AC12">
         <f ca="1" t="shared" si="7"/>
-        <v>219</v>
+        <v>168</v>
       </c>
       <c r="AD12">
         <f ca="1" t="shared" si="7"/>
-        <v>131</v>
+        <v>112</v>
       </c>
       <c r="AE12">
         <f ca="1" t="shared" si="7"/>
-        <v>213</v>
+        <v>84</v>
       </c>
     </row>
     <row r="13" spans="1:31">
@@ -2272,44 +2272,44 @@
         <v>2</v>
       </c>
       <c r="B17">
-        <f ca="1" t="shared" ref="B17:AE17" si="8">IF(B18*3&gt;B19,B18*3-B19,0)</f>
+        <f ca="1" t="shared" ref="B17:AE17" si="8">IF(C18*3&gt;B19,C18*3-B19,0)</f>
         <v>0</v>
       </c>
       <c r="C17">
         <f ca="1" t="shared" si="8"/>
-        <v>302</v>
+        <v>130</v>
       </c>
       <c r="D17">
         <f ca="1" t="shared" si="8"/>
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="E17">
         <f ca="1" t="shared" si="8"/>
-        <v>0</v>
+        <v>132</v>
       </c>
       <c r="F17">
         <f ca="1" t="shared" si="8"/>
-        <v>0</v>
+        <v>54</v>
       </c>
       <c r="G17">
         <f ca="1" t="shared" si="8"/>
-        <v>93</v>
+        <v>72</v>
       </c>
       <c r="H17">
         <f ca="1" t="shared" si="8"/>
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="I17">
         <f ca="1" t="shared" si="8"/>
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="J17">
         <f ca="1" t="shared" si="8"/>
-        <v>0</v>
+        <v>197</v>
       </c>
       <c r="K17">
         <f ca="1" t="shared" si="8"/>
-        <v>265</v>
+        <v>0</v>
       </c>
       <c r="L17">
         <f ca="1" t="shared" si="8"/>
@@ -2317,19 +2317,19 @@
       </c>
       <c r="M17">
         <f ca="1" t="shared" si="8"/>
-        <v>56</v>
+        <v>173</v>
       </c>
       <c r="N17">
         <f ca="1" t="shared" si="8"/>
-        <v>140</v>
+        <v>43</v>
       </c>
       <c r="O17">
         <f ca="1" t="shared" si="8"/>
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="P17">
         <f ca="1" t="shared" si="8"/>
-        <v>178</v>
+        <v>0</v>
       </c>
       <c r="Q17">
         <f ca="1" t="shared" si="8"/>
@@ -2341,35 +2341,35 @@
       </c>
       <c r="S17">
         <f ca="1" t="shared" si="8"/>
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="T17">
         <f ca="1" t="shared" si="8"/>
-        <v>0</v>
+        <v>54</v>
       </c>
       <c r="U17">
         <f ca="1" t="shared" si="8"/>
-        <v>0</v>
+        <v>96</v>
       </c>
       <c r="V17">
         <f ca="1" t="shared" si="8"/>
-        <v>154</v>
+        <v>120</v>
       </c>
       <c r="W17">
         <f ca="1" t="shared" si="8"/>
+        <v>40</v>
+      </c>
+      <c r="X17">
+        <f ca="1" t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="Y17">
+        <f ca="1" t="shared" si="8"/>
         <v>5</v>
       </c>
-      <c r="X17">
-        <f ca="1" t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="Y17">
-        <f ca="1" t="shared" si="8"/>
-        <v>7</v>
-      </c>
       <c r="Z17">
         <f ca="1" t="shared" si="8"/>
-        <v>0</v>
+        <v>191</v>
       </c>
       <c r="AA17">
         <f ca="1" t="shared" si="8"/>
@@ -2377,15 +2377,15 @@
       </c>
       <c r="AB17">
         <f ca="1" t="shared" si="8"/>
-        <v>141</v>
+        <v>0</v>
       </c>
       <c r="AC17">
         <f ca="1" t="shared" si="8"/>
-        <v>0</v>
+        <v>59</v>
       </c>
       <c r="AD17">
         <f ca="1" t="shared" si="8"/>
-        <v>80</v>
+        <v>190</v>
       </c>
       <c r="AE17">
         <f ca="1" t="shared" si="8"/>
@@ -2398,123 +2398,123 @@
       </c>
       <c r="B18">
         <f ca="1" t="shared" ref="B18:AE18" si="9">RANDBETWEEN(10,100)</f>
-        <v>13</v>
+        <v>51</v>
       </c>
       <c r="C18">
         <f ca="1" t="shared" si="9"/>
-        <v>99</v>
+        <v>26</v>
       </c>
       <c r="D18">
         <f ca="1" t="shared" si="9"/>
-        <v>80</v>
+        <v>66</v>
       </c>
       <c r="E18">
         <f ca="1" t="shared" si="9"/>
+        <v>21</v>
+      </c>
+      <c r="F18">
+        <f ca="1" t="shared" si="9"/>
+        <v>81</v>
+      </c>
+      <c r="G18">
+        <f ca="1" t="shared" si="9"/>
+        <v>72</v>
+      </c>
+      <c r="H18">
+        <f ca="1" t="shared" si="9"/>
+        <v>72</v>
+      </c>
+      <c r="I18">
+        <f ca="1" t="shared" si="9"/>
+        <v>27</v>
+      </c>
+      <c r="J18">
+        <f ca="1" t="shared" si="9"/>
         <v>14</v>
       </c>
-      <c r="F18">
+      <c r="K18">
+        <f ca="1" t="shared" si="9"/>
+        <v>100</v>
+      </c>
+      <c r="L18">
+        <f ca="1" t="shared" si="9"/>
+        <v>24</v>
+      </c>
+      <c r="M18">
+        <f ca="1" t="shared" si="9"/>
+        <v>49</v>
+      </c>
+      <c r="N18">
+        <f ca="1" t="shared" si="9"/>
+        <v>100</v>
+      </c>
+      <c r="O18">
+        <f ca="1" t="shared" si="9"/>
+        <v>81</v>
+      </c>
+      <c r="P18">
+        <f ca="1" t="shared" si="9"/>
+        <v>84</v>
+      </c>
+      <c r="Q18">
+        <f ca="1" t="shared" si="9"/>
+        <v>27</v>
+      </c>
+      <c r="R18">
+        <f ca="1" t="shared" si="9"/>
+        <v>37</v>
+      </c>
+      <c r="S18">
+        <f ca="1" t="shared" si="9"/>
+        <v>18</v>
+      </c>
+      <c r="T18">
+        <f ca="1" t="shared" si="9"/>
+        <v>63</v>
+      </c>
+      <c r="U18">
+        <f ca="1" t="shared" si="9"/>
+        <v>60</v>
+      </c>
+      <c r="V18">
+        <f ca="1" t="shared" si="9"/>
+        <v>72</v>
+      </c>
+      <c r="W18">
+        <f ca="1" t="shared" si="9"/>
+        <v>88</v>
+      </c>
+      <c r="X18">
+        <f ca="1" t="shared" si="9"/>
+        <v>72</v>
+      </c>
+      <c r="Y18">
+        <f ca="1" t="shared" si="9"/>
+        <v>26</v>
+      </c>
+      <c r="Z18">
+        <f ca="1" t="shared" si="9"/>
+        <v>41</v>
+      </c>
+      <c r="AA18">
+        <f ca="1" t="shared" si="9"/>
+        <v>91</v>
+      </c>
+      <c r="AB18">
+        <f ca="1" t="shared" si="9"/>
+        <v>42</v>
+      </c>
+      <c r="AC18">
+        <f ca="1" t="shared" si="9"/>
+        <v>34</v>
+      </c>
+      <c r="AD18">
         <f ca="1" t="shared" si="9"/>
         <v>55</v>
       </c>
-      <c r="G18">
-        <f ca="1" t="shared" si="9"/>
-        <v>66</v>
-      </c>
-      <c r="H18">
-        <f ca="1" t="shared" si="9"/>
-        <v>56</v>
-      </c>
-      <c r="I18">
-        <f ca="1" t="shared" si="9"/>
-        <v>50</v>
-      </c>
-      <c r="J18">
-        <f ca="1" t="shared" si="9"/>
-        <v>35</v>
-      </c>
-      <c r="K18">
-        <f ca="1" t="shared" si="9"/>
-        <v>95</v>
-      </c>
-      <c r="L18">
-        <f ca="1" t="shared" si="9"/>
-        <v>53</v>
-      </c>
-      <c r="M18">
-        <f ca="1" t="shared" si="9"/>
-        <v>72</v>
-      </c>
-      <c r="N18">
-        <f ca="1" t="shared" si="9"/>
-        <v>89</v>
-      </c>
-      <c r="O18">
-        <f ca="1" t="shared" si="9"/>
-        <v>57</v>
-      </c>
-      <c r="P18">
-        <f ca="1" t="shared" si="9"/>
-        <v>97</v>
-      </c>
-      <c r="Q18">
-        <f ca="1" t="shared" si="9"/>
-        <v>69</v>
-      </c>
-      <c r="R18">
-        <f ca="1" t="shared" si="9"/>
-        <v>17</v>
-      </c>
-      <c r="S18">
-        <f ca="1" t="shared" si="9"/>
-        <v>75</v>
-      </c>
-      <c r="T18">
-        <f ca="1" t="shared" si="9"/>
-        <v>14</v>
-      </c>
-      <c r="U18">
-        <f ca="1" t="shared" si="9"/>
-        <v>41</v>
-      </c>
-      <c r="V18">
-        <f ca="1" t="shared" si="9"/>
-        <v>81</v>
-      </c>
-      <c r="W18">
-        <f ca="1" t="shared" si="9"/>
-        <v>62</v>
-      </c>
-      <c r="X18">
-        <f ca="1" t="shared" si="9"/>
-        <v>21</v>
-      </c>
-      <c r="Y18">
-        <f ca="1" t="shared" si="9"/>
-        <v>43</v>
-      </c>
-      <c r="Z18">
-        <f ca="1" t="shared" si="9"/>
-        <v>14</v>
-      </c>
-      <c r="AA18">
-        <f ca="1" t="shared" si="9"/>
-        <v>20</v>
-      </c>
-      <c r="AB18">
-        <f ca="1" t="shared" si="9"/>
-        <v>59</v>
-      </c>
-      <c r="AC18">
-        <f ca="1" t="shared" si="9"/>
-        <v>21</v>
-      </c>
-      <c r="AD18">
-        <f ca="1" t="shared" si="9"/>
-        <v>59</v>
-      </c>
       <c r="AE18">
         <f ca="1" t="shared" si="9"/>
-        <v>11</v>
+        <v>100</v>
       </c>
     </row>
     <row r="19" spans="1:31">
@@ -2526,119 +2526,119 @@
       </c>
       <c r="C19">
         <f ca="1" t="shared" ref="C19:AE19" si="10">B19-C18+B17</f>
-        <v>-5</v>
+        <v>68</v>
       </c>
       <c r="D19">
         <f ca="1" t="shared" si="10"/>
-        <v>217</v>
+        <v>132</v>
       </c>
       <c r="E19">
         <f ca="1" t="shared" si="10"/>
-        <v>226</v>
+        <v>111</v>
       </c>
       <c r="F19">
         <f ca="1" t="shared" si="10"/>
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="G19">
         <f ca="1" t="shared" si="10"/>
-        <v>105</v>
+        <v>144</v>
       </c>
       <c r="H19">
         <f ca="1" t="shared" si="10"/>
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="I19">
         <f ca="1" t="shared" si="10"/>
+        <v>117</v>
+      </c>
+      <c r="J19">
+        <f ca="1" t="shared" si="10"/>
+        <v>103</v>
+      </c>
+      <c r="K19">
+        <f ca="1" t="shared" si="10"/>
+        <v>200</v>
+      </c>
+      <c r="L19">
+        <f ca="1" t="shared" si="10"/>
+        <v>176</v>
+      </c>
+      <c r="M19">
+        <f ca="1" t="shared" si="10"/>
+        <v>127</v>
+      </c>
+      <c r="N19">
+        <f ca="1" t="shared" si="10"/>
+        <v>200</v>
+      </c>
+      <c r="O19">
+        <f ca="1" t="shared" si="10"/>
+        <v>162</v>
+      </c>
+      <c r="P19">
+        <f ca="1" t="shared" si="10"/>
+        <v>168</v>
+      </c>
+      <c r="Q19">
+        <f ca="1" t="shared" si="10"/>
+        <v>141</v>
+      </c>
+      <c r="R19">
+        <f ca="1" t="shared" si="10"/>
+        <v>104</v>
+      </c>
+      <c r="S19">
+        <f ca="1" t="shared" si="10"/>
+        <v>86</v>
+      </c>
+      <c r="T19">
+        <f ca="1" t="shared" si="10"/>
+        <v>126</v>
+      </c>
+      <c r="U19">
+        <f ca="1" t="shared" si="10"/>
+        <v>120</v>
+      </c>
+      <c r="V19">
+        <f ca="1" t="shared" si="10"/>
+        <v>144</v>
+      </c>
+      <c r="W19">
+        <f ca="1" t="shared" si="10"/>
+        <v>176</v>
+      </c>
+      <c r="X19">
+        <f ca="1" t="shared" si="10"/>
+        <v>144</v>
+      </c>
+      <c r="Y19">
+        <f ca="1" t="shared" si="10"/>
         <v>118</v>
       </c>
-      <c r="J19">
-        <f ca="1" t="shared" si="10"/>
-        <v>115</v>
-      </c>
-      <c r="K19">
-        <f ca="1" t="shared" si="10"/>
-        <v>20</v>
-      </c>
-      <c r="L19">
-        <f ca="1" t="shared" si="10"/>
-        <v>232</v>
-      </c>
-      <c r="M19">
-        <f ca="1" t="shared" si="10"/>
-        <v>160</v>
-      </c>
-      <c r="N19">
-        <f ca="1" t="shared" si="10"/>
-        <v>127</v>
-      </c>
-      <c r="O19">
-        <f ca="1" t="shared" si="10"/>
-        <v>210</v>
-      </c>
-      <c r="P19">
-        <f ca="1" t="shared" si="10"/>
-        <v>113</v>
-      </c>
-      <c r="Q19">
-        <f ca="1" t="shared" si="10"/>
-        <v>222</v>
-      </c>
-      <c r="R19">
-        <f ca="1" t="shared" si="10"/>
-        <v>205</v>
-      </c>
-      <c r="S19">
-        <f ca="1" t="shared" si="10"/>
-        <v>130</v>
-      </c>
-      <c r="T19">
-        <f ca="1" t="shared" si="10"/>
-        <v>211</v>
-      </c>
-      <c r="U19">
-        <f ca="1" t="shared" si="10"/>
-        <v>170</v>
-      </c>
-      <c r="V19">
-        <f ca="1" t="shared" si="10"/>
-        <v>89</v>
-      </c>
-      <c r="W19">
-        <f ca="1" t="shared" si="10"/>
-        <v>181</v>
-      </c>
-      <c r="X19">
-        <f ca="1" t="shared" si="10"/>
-        <v>165</v>
-      </c>
-      <c r="Y19">
-        <f ca="1" t="shared" si="10"/>
-        <v>122</v>
-      </c>
       <c r="Z19">
         <f ca="1" t="shared" si="10"/>
-        <v>115</v>
+        <v>82</v>
       </c>
       <c r="AA19">
         <f ca="1" t="shared" si="10"/>
-        <v>95</v>
+        <v>182</v>
       </c>
       <c r="AB19">
         <f ca="1" t="shared" si="10"/>
-        <v>36</v>
+        <v>140</v>
       </c>
       <c r="AC19">
         <f ca="1" t="shared" si="10"/>
-        <v>156</v>
+        <v>106</v>
       </c>
       <c r="AD19">
         <f ca="1" t="shared" si="10"/>
-        <v>97</v>
+        <v>110</v>
       </c>
       <c r="AE19">
         <f ca="1" t="shared" si="10"/>
-        <v>166</v>
+        <v>200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>